<commit_message>
Medição Agrupada Atualizada 27/10
</commit_message>
<xml_diff>
--- a/Taxa de Crescimento.xlsx
+++ b/Taxa de Crescimento.xlsx
@@ -1602,7 +1602,7 @@
         <v>12165</v>
       </c>
       <c r="P16" t="n">
-        <v>11584</v>
+        <v>13113</v>
       </c>
       <c r="Q16" t="n">
         <v>14496</v>
@@ -1681,7 +1681,7 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>299</v>
       </c>
       <c r="Q17" t="n">
         <v>4925</v>
@@ -1760,7 +1760,7 @@
         <v>14925</v>
       </c>
       <c r="P18" t="n">
-        <v>13690</v>
+        <v>14574</v>
       </c>
       <c r="Q18" t="n">
         <v>28370</v>
@@ -3965,13 +3965,13 @@
         <v>1625</v>
       </c>
       <c r="P49" t="n">
-        <v>1649</v>
+        <v>1724</v>
       </c>
       <c r="Q49" t="n">
-        <v>1649</v>
+        <v>1724</v>
       </c>
       <c r="R49" t="n">
-        <v>54.97</v>
+        <v>57.47</v>
       </c>
       <c r="S49" t="n">
         <v>8</v>
@@ -3985,10 +3985,10 @@
         <v>1478.58</v>
       </c>
       <c r="V49" t="n">
-        <v>11.53</v>
+        <v>16.6</v>
       </c>
       <c r="W49" t="n">
-        <v>1.225986747431812</v>
+        <v>1.263792209863485</v>
       </c>
     </row>
     <row r="50">
@@ -4168,13 +4168,13 @@
         <v>2639</v>
       </c>
       <c r="P52" t="n">
-        <v>2701</v>
+        <v>2776</v>
       </c>
       <c r="Q52" t="n">
-        <v>2726</v>
+        <v>2776</v>
       </c>
       <c r="R52" t="n">
-        <v>10.9</v>
+        <v>11.1</v>
       </c>
       <c r="S52" t="n">
         <v>8</v>
@@ -4188,7 +4188,7 @@
         <v>2979.35</v>
       </c>
       <c r="V52" t="n">
-        <v>-8.5</v>
+        <v>-6.83</v>
       </c>
       <c r="W52" t="inlineStr"/>
     </row>
@@ -6143,13 +6143,13 @@
         <v>19559</v>
       </c>
       <c r="P79" t="n">
-        <v>20590</v>
+        <v>22207</v>
       </c>
       <c r="Q79" t="n">
-        <v>20590</v>
+        <v>22207</v>
       </c>
       <c r="R79" t="n">
-        <v>45.76</v>
+        <v>49.35</v>
       </c>
       <c r="S79" t="n">
         <v>8</v>
@@ -6163,10 +6163,10 @@
         <v>19321.81</v>
       </c>
       <c r="V79" t="n">
-        <v>6.56</v>
+        <v>14.93</v>
       </c>
       <c r="W79" t="n">
-        <v>1.169702235577781</v>
+        <v>1.252674732161622</v>
       </c>
     </row>
     <row r="80">
@@ -6376,13 +6376,13 @@
         <v>36867</v>
       </c>
       <c r="P82" t="n">
-        <v>38477</v>
+        <v>38755</v>
       </c>
       <c r="Q82" t="n">
-        <v>38477</v>
+        <v>38755</v>
       </c>
       <c r="R82" t="n">
-        <v>85.5</v>
+        <v>86.12</v>
       </c>
       <c r="S82" t="n">
         <v>8</v>
@@ -6396,10 +6396,10 @@
         <v>35969.29</v>
       </c>
       <c r="V82" t="n">
-        <v>6.97</v>
+        <v>7.74</v>
       </c>
       <c r="W82" t="n">
-        <v>1.175626584341361</v>
+        <v>1.185937349296872</v>
       </c>
     </row>
     <row r="83">
@@ -8231,7 +8231,7 @@
         <v>27513</v>
       </c>
       <c r="P107" t="n">
-        <v>14564</v>
+        <v>13866</v>
       </c>
       <c r="Q107" t="n">
         <v>27513</v>
@@ -8310,7 +8310,7 @@
         <v>9607</v>
       </c>
       <c r="P108" t="n">
-        <v>3680</v>
+        <v>3616</v>
       </c>
       <c r="Q108" t="n">
         <v>9607</v>
@@ -8688,13 +8688,13 @@
         <v>11434</v>
       </c>
       <c r="P114" t="n">
-        <v>11485</v>
+        <v>11521</v>
       </c>
       <c r="Q114" t="n">
-        <v>11485</v>
+        <v>11521</v>
       </c>
       <c r="R114" t="n">
-        <v>91.88</v>
+        <v>92.17</v>
       </c>
       <c r="S114" t="n">
         <v>8</v>
@@ -8708,7 +8708,7 @@
         <v>11732.5</v>
       </c>
       <c r="V114" t="n">
-        <v>-2.11</v>
+        <v>-1.8</v>
       </c>
       <c r="W114" t="inlineStr"/>
     </row>
@@ -11929,7 +11929,7 @@
         <v>19750</v>
       </c>
       <c r="P159" t="n">
-        <v>18791</v>
+        <v>19637</v>
       </c>
       <c r="Q159" t="n">
         <v>19750</v>
@@ -15792,13 +15792,13 @@
         <v>22450</v>
       </c>
       <c r="P212" t="n">
-        <v>0</v>
+        <v>23928</v>
       </c>
       <c r="Q212" t="n">
-        <v>22789</v>
+        <v>23928</v>
       </c>
       <c r="R212" t="n">
-        <v>91.16</v>
+        <v>95.70999999999999</v>
       </c>
       <c r="S212" t="n">
         <v>8</v>
@@ -15812,10 +15812,10 @@
         <v>7305</v>
       </c>
       <c r="V212" t="n">
-        <v>211.96</v>
+        <v>227.56</v>
       </c>
       <c r="W212" t="n">
-        <v>1.562624008317012</v>
+        <v>1.571899082385014</v>
       </c>
     </row>
     <row r="213">
@@ -15973,13 +15973,13 @@
         <v>2584</v>
       </c>
       <c r="P215" t="n">
-        <v>2639</v>
+        <v>2828</v>
       </c>
       <c r="Q215" t="n">
-        <v>2639</v>
+        <v>2828</v>
       </c>
       <c r="R215" t="n">
-        <v>87.97</v>
+        <v>94.27</v>
       </c>
       <c r="S215" t="n">
         <v>8</v>
@@ -15993,10 +15993,10 @@
         <v>2510.67</v>
       </c>
       <c r="V215" t="n">
-        <v>5.11</v>
+        <v>12.64</v>
       </c>
       <c r="W215" t="n">
-        <v>1.145605460470037</v>
+        <v>1.23541325358259</v>
       </c>
     </row>
     <row r="216">
@@ -16443,13 +16443,13 @@
         <v>4639</v>
       </c>
       <c r="P221" t="n">
-        <v>4878</v>
+        <v>5240</v>
       </c>
       <c r="Q221" t="n">
-        <v>4878</v>
+        <v>5240</v>
       </c>
       <c r="R221" t="n">
-        <v>52.03</v>
+        <v>55.89</v>
       </c>
       <c r="S221" t="n">
         <v>8</v>
@@ -16463,7 +16463,7 @@
         <v>5598.92</v>
       </c>
       <c r="V221" t="n">
-        <v>-12.88</v>
+        <v>-6.41</v>
       </c>
       <c r="W221" t="inlineStr"/>
     </row>
@@ -19153,7 +19153,7 @@
         <v>1797</v>
       </c>
       <c r="P257" t="n">
-        <v>1220</v>
+        <v>1215</v>
       </c>
       <c r="Q257" t="n">
         <v>1930</v>
@@ -20097,7 +20097,7 @@
         <v>5986</v>
       </c>
       <c r="P269" t="n">
-        <v>4716</v>
+        <v>5695</v>
       </c>
       <c r="Q269" t="n">
         <v>7429</v>
@@ -23271,13 +23271,13 @@
         <v>6140</v>
       </c>
       <c r="P311" t="n">
-        <v>6016</v>
+        <v>6267</v>
       </c>
       <c r="Q311" t="n">
-        <v>6140</v>
+        <v>6267</v>
       </c>
       <c r="R311" t="n">
-        <v>61.4</v>
+        <v>62.67</v>
       </c>
       <c r="S311" t="n">
         <v>8</v>
@@ -23291,10 +23291,10 @@
         <v>4483.32</v>
       </c>
       <c r="V311" t="n">
-        <v>36.95</v>
+        <v>39.78</v>
       </c>
       <c r="W311" t="n">
-        <v>1.350935259341024</v>
+        <v>1.359268955881436</v>
       </c>
     </row>
     <row r="312">
@@ -23427,13 +23427,13 @@
         <v>3754</v>
       </c>
       <c r="P313" t="n">
-        <v>3843</v>
+        <v>4124</v>
       </c>
       <c r="Q313" t="n">
-        <v>3843</v>
+        <v>4124</v>
       </c>
       <c r="R313" t="n">
-        <v>38.43</v>
+        <v>41.24</v>
       </c>
       <c r="S313" t="n">
         <v>8</v>
@@ -23447,7 +23447,7 @@
         <v>4882.03</v>
       </c>
       <c r="V313" t="n">
-        <v>-21.28</v>
+        <v>-15.53</v>
       </c>
       <c r="W313" t="inlineStr"/>
     </row>
@@ -24434,7 +24434,7 @@
         <v>1176</v>
       </c>
       <c r="P328" t="n">
-        <v>1366</v>
+        <v>1450</v>
       </c>
       <c r="Q328" t="n">
         <v>1637</v>
@@ -25109,13 +25109,13 @@
         <v>5311</v>
       </c>
       <c r="P337" t="n">
-        <v>4993</v>
+        <v>6185</v>
       </c>
       <c r="Q337" t="n">
-        <v>5311</v>
+        <v>6185</v>
       </c>
       <c r="R337" t="n">
-        <v>44.26</v>
+        <v>51.54</v>
       </c>
       <c r="S337" t="n">
         <v>8</v>
@@ -25129,10 +25129,10 @@
         <v>4336.29</v>
       </c>
       <c r="V337" t="n">
-        <v>22.48</v>
+        <v>42.63</v>
       </c>
       <c r="W337" t="n">
-        <v>1.296133370647445</v>
+        <v>1.367129362810221</v>
       </c>
     </row>
     <row r="338">
@@ -26271,7 +26271,7 @@
         <v>3755</v>
       </c>
       <c r="P353" t="n">
-        <v>3672</v>
+        <v>3753</v>
       </c>
       <c r="Q353" t="n">
         <v>3782</v>
@@ -26662,13 +26662,13 @@
         <v>1958</v>
       </c>
       <c r="P358" t="n">
-        <v>2096</v>
+        <v>2270</v>
       </c>
       <c r="Q358" t="n">
-        <v>2096</v>
+        <v>2270</v>
       </c>
       <c r="R358" t="n">
-        <v>20.96</v>
+        <v>22.7</v>
       </c>
       <c r="S358" t="n">
         <v>8</v>
@@ -26682,9 +26682,11 @@
         <v>2182.6</v>
       </c>
       <c r="V358" t="n">
-        <v>-3.97</v>
-      </c>
-      <c r="W358" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="W358" t="n">
+        <v>1.122462048309373</v>
+      </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -27515,7 +27517,7 @@
         <v>6493</v>
       </c>
       <c r="P369" t="n">
-        <v>6433</v>
+        <v>6490</v>
       </c>
       <c r="Q369" t="n">
         <v>6493</v>
@@ -29229,7 +29231,7 @@
         <v>2537</v>
       </c>
       <c r="P391" t="n">
-        <v>2442</v>
+        <v>2486</v>
       </c>
       <c r="Q391" t="n">
         <v>2537</v>
@@ -29306,7 +29308,7 @@
         <v>7403</v>
       </c>
       <c r="P392" t="n">
-        <v>6727</v>
+        <v>6105</v>
       </c>
       <c r="Q392" t="n">
         <v>7403</v>
@@ -30601,13 +30603,13 @@
         <v>875</v>
       </c>
       <c r="P409" t="n">
-        <v>1504</v>
+        <v>1469</v>
       </c>
       <c r="Q409" t="n">
-        <v>1504</v>
+        <v>1469</v>
       </c>
       <c r="R409" t="n">
-        <v>8.85</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="S409" t="n">
         <v>8</v>
@@ -30621,7 +30623,7 @@
         <v>1512.99</v>
       </c>
       <c r="V409" t="n">
-        <v>-0.59</v>
+        <v>-2.91</v>
       </c>
       <c r="W409" t="inlineStr"/>
     </row>
@@ -31221,7 +31223,7 @@
         <v>7301</v>
       </c>
       <c r="P417" t="n">
-        <v>7004</v>
+        <v>7063</v>
       </c>
       <c r="Q417" t="n">
         <v>7501</v>
@@ -32313,13 +32315,13 @@
         <v>5628</v>
       </c>
       <c r="P431" t="n">
-        <v>5869</v>
+        <v>6049</v>
       </c>
       <c r="Q431" t="n">
-        <v>5869</v>
+        <v>6049</v>
       </c>
       <c r="R431" t="n">
-        <v>58.69</v>
+        <v>60.49</v>
       </c>
       <c r="S431" t="n">
         <v>8</v>
@@ -32333,7 +32335,7 @@
         <v>8447.5</v>
       </c>
       <c r="V431" t="n">
-        <v>-30.52</v>
+        <v>-28.39</v>
       </c>
       <c r="W431" t="inlineStr"/>
     </row>
@@ -33948,13 +33950,13 @@
         <v>4114</v>
       </c>
       <c r="P452" t="n">
-        <v>5106</v>
+        <v>5598</v>
       </c>
       <c r="Q452" t="n">
-        <v>5106</v>
+        <v>5598</v>
       </c>
       <c r="R452" t="n">
-        <v>51.06</v>
+        <v>55.98</v>
       </c>
       <c r="S452" t="n">
         <v>8</v>
@@ -33968,10 +33970,10 @@
         <v>4416.41</v>
       </c>
       <c r="V452" t="n">
-        <v>15.61</v>
+        <v>26.75</v>
       </c>
       <c r="W452" t="n">
-        <v>1.257332790719738</v>
+        <v>1.315054188517107</v>
       </c>
     </row>
     <row r="453">
@@ -34880,7 +34882,7 @@
         <v>5366</v>
       </c>
       <c r="P464" t="n">
-        <v>3176</v>
+        <v>4367</v>
       </c>
       <c r="Q464" t="n">
         <v>5366</v>
@@ -34957,13 +34959,13 @@
         <v>525</v>
       </c>
       <c r="P465" t="n">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="Q465" t="n">
-        <v>578</v>
+        <v>586</v>
       </c>
       <c r="R465" t="n">
-        <v>28.9</v>
+        <v>29.3</v>
       </c>
       <c r="S465" t="n">
         <v>8</v>
@@ -34977,7 +34979,7 @@
         <v>620.76</v>
       </c>
       <c r="V465" t="n">
-        <v>-6.89</v>
+        <v>-5.6</v>
       </c>
       <c r="W465" t="inlineStr"/>
     </row>
@@ -36355,7 +36357,7 @@
         <v>8975</v>
       </c>
       <c r="P483" t="n">
-        <v>8897</v>
+        <v>8942</v>
       </c>
       <c r="Q483" t="n">
         <v>8975</v>
@@ -37058,13 +37060,13 @@
         <v>4966</v>
       </c>
       <c r="P492" t="n">
-        <v>5269</v>
+        <v>5379</v>
       </c>
       <c r="Q492" t="n">
-        <v>5269</v>
+        <v>5379</v>
       </c>
       <c r="R492" t="n">
-        <v>52.69</v>
+        <v>53.79</v>
       </c>
       <c r="S492" t="n">
         <v>8</v>
@@ -37078,10 +37080,10 @@
         <v>4910.37</v>
       </c>
       <c r="V492" t="n">
-        <v>7.3</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="W492" t="n">
-        <v>1.180167285354979</v>
+        <v>1.206782576531111</v>
       </c>
     </row>
     <row r="493">
@@ -37370,13 +37372,13 @@
         <v>4717</v>
       </c>
       <c r="P496" t="n">
-        <v>4727</v>
+        <v>4744</v>
       </c>
       <c r="Q496" t="n">
-        <v>4727</v>
+        <v>4744</v>
       </c>
       <c r="R496" t="n">
-        <v>47.09</v>
+        <v>47.26</v>
       </c>
       <c r="S496" t="n">
         <v>8</v>
@@ -37390,10 +37392,10 @@
         <v>4343.4</v>
       </c>
       <c r="V496" t="n">
-        <v>8.83</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="W496" t="n">
-        <v>1.199030025541241</v>
+        <v>1.203356320573685</v>
       </c>
     </row>
     <row r="497">
@@ -37994,7 +37996,7 @@
         <v>3660</v>
       </c>
       <c r="P504" t="n">
-        <v>3555</v>
+        <v>3569</v>
       </c>
       <c r="Q504" t="n">
         <v>3660</v>
@@ -38460,13 +38462,13 @@
         <v>2776</v>
       </c>
       <c r="P510" t="n">
-        <v>3336</v>
+        <v>3344</v>
       </c>
       <c r="Q510" t="n">
-        <v>3336</v>
+        <v>3344</v>
       </c>
       <c r="R510" t="n">
-        <v>33.36</v>
+        <v>33.44</v>
       </c>
       <c r="S510" t="n">
         <v>8</v>
@@ -38480,7 +38482,7 @@
         <v>6017.96</v>
       </c>
       <c r="V510" t="n">
-        <v>-44.57</v>
+        <v>-44.43</v>
       </c>
       <c r="W510" t="inlineStr"/>
     </row>
@@ -39157,7 +39159,7 @@
         <v>5093</v>
       </c>
       <c r="P519" t="n">
-        <v>4880</v>
+        <v>4911</v>
       </c>
       <c r="Q519" t="n">
         <v>5093</v>
@@ -39623,13 +39625,13 @@
         <v>6020</v>
       </c>
       <c r="P525" t="n">
-        <v>5940</v>
+        <v>6033</v>
       </c>
       <c r="Q525" t="n">
-        <v>6020</v>
+        <v>6033</v>
       </c>
       <c r="R525" t="n">
-        <v>60.2</v>
+        <v>60.33</v>
       </c>
       <c r="S525" t="n">
         <v>8</v>
@@ -39643,7 +39645,7 @@
         <v>8209.059999999999</v>
       </c>
       <c r="V525" t="n">
-        <v>-26.67</v>
+        <v>-26.51</v>
       </c>
       <c r="W525" t="inlineStr"/>
     </row>
@@ -40468,13 +40470,13 @@
         <v>665</v>
       </c>
       <c r="P536" t="n">
-        <v>657</v>
+        <v>919</v>
       </c>
       <c r="Q536" t="n">
-        <v>707</v>
+        <v>919</v>
       </c>
       <c r="R536" t="n">
-        <v>35.35</v>
+        <v>45.95</v>
       </c>
       <c r="S536" t="n">
         <v>8</v>
@@ -40488,7 +40490,7 @@
         <v>1663.67</v>
       </c>
       <c r="V536" t="n">
-        <v>-57.5</v>
+        <v>-44.76</v>
       </c>
       <c r="W536" t="inlineStr"/>
     </row>
@@ -41237,7 +41239,7 @@
         <v>5417</v>
       </c>
       <c r="P547" t="n">
-        <v>2691</v>
+        <v>2663</v>
       </c>
       <c r="Q547" t="n">
         <v>6510</v>
@@ -41314,7 +41316,7 @@
         <v>6861</v>
       </c>
       <c r="P548" t="n">
-        <v>2531</v>
+        <v>2427</v>
       </c>
       <c r="Q548" t="n">
         <v>6861</v>
@@ -42517,7 +42519,7 @@
         <v>4348</v>
       </c>
       <c r="P565" t="n">
-        <v>3938</v>
+        <v>4224</v>
       </c>
       <c r="Q565" t="n">
         <v>4348</v>
@@ -43192,13 +43194,13 @@
         <v>5101</v>
       </c>
       <c r="P574" t="n">
-        <v>5939</v>
+        <v>6088</v>
       </c>
       <c r="Q574" t="n">
-        <v>5939</v>
+        <v>6088</v>
       </c>
       <c r="R574" t="n">
-        <v>84.84</v>
+        <v>86.97</v>
       </c>
       <c r="S574" t="n">
         <v>8</v>
@@ -43212,10 +43214,10 @@
         <v>5121.94</v>
       </c>
       <c r="V574" t="n">
-        <v>15.95</v>
+        <v>18.86</v>
       </c>
       <c r="W574" t="n">
-        <v>1.259592474573147</v>
+        <v>1.277306554312118</v>
       </c>
     </row>
     <row r="575">
@@ -44408,7 +44410,7 @@
         <v>2423</v>
       </c>
       <c r="P590" t="n">
-        <v>1213</v>
+        <v>1970</v>
       </c>
       <c r="Q590" t="n">
         <v>3670</v>
@@ -44793,7 +44795,7 @@
         <v>398</v>
       </c>
       <c r="P595" t="n">
-        <v>398</v>
+        <v>349</v>
       </c>
       <c r="Q595" t="n">
         <v>398</v>
@@ -48394,7 +48396,7 @@
         <v>7734</v>
       </c>
       <c r="P642" t="n">
-        <v>7157</v>
+        <v>7593</v>
       </c>
       <c r="Q642" t="n">
         <v>8193</v>
@@ -49837,7 +49839,7 @@
         <v>8291</v>
       </c>
       <c r="P661" t="n">
-        <v>6230</v>
+        <v>7026</v>
       </c>
       <c r="Q661" t="n">
         <v>9245</v>
@@ -52970,13 +52972,13 @@
         <v>6744</v>
       </c>
       <c r="P702" t="n">
-        <v>6642</v>
+        <v>6882</v>
       </c>
       <c r="Q702" t="n">
-        <v>6813</v>
+        <v>6882</v>
       </c>
       <c r="R702" t="n">
-        <v>68.13</v>
+        <v>68.81999999999999</v>
       </c>
       <c r="S702" t="n">
         <v>8</v>
@@ -52990,7 +52992,7 @@
         <v>9010.68</v>
       </c>
       <c r="V702" t="n">
-        <v>-24.39</v>
+        <v>-23.62</v>
       </c>
       <c r="W702" t="inlineStr"/>
     </row>
@@ -53201,13 +53203,13 @@
         <v>2843</v>
       </c>
       <c r="P705" t="n">
-        <v>2940</v>
+        <v>2632</v>
       </c>
       <c r="Q705" t="n">
-        <v>2940</v>
+        <v>2843</v>
       </c>
       <c r="R705" t="n">
-        <v>42</v>
+        <v>40.61</v>
       </c>
       <c r="S705" t="n">
         <v>8</v>
@@ -53221,11 +53223,9 @@
         <v>2866.48</v>
       </c>
       <c r="V705" t="n">
-        <v>2.56</v>
-      </c>
-      <c r="W705" t="n">
-        <v>1.081483747120199</v>
-      </c>
+        <v>-0.82</v>
+      </c>
+      <c r="W705" t="inlineStr"/>
     </row>
     <row r="706">
       <c r="A706" t="inlineStr">
@@ -55454,7 +55454,7 @@
         <v>6867</v>
       </c>
       <c r="P734" t="n">
-        <v>6273</v>
+        <v>6286</v>
       </c>
       <c r="Q734" t="n">
         <v>7742</v>
@@ -55841,13 +55841,13 @@
         <v>7507</v>
       </c>
       <c r="P739" t="n">
-        <v>7521</v>
+        <v>7604</v>
       </c>
       <c r="Q739" t="n">
-        <v>7577</v>
+        <v>7604</v>
       </c>
       <c r="R739" t="n">
-        <v>75.48</v>
+        <v>75.73999999999999</v>
       </c>
       <c r="S739" t="n">
         <v>8</v>
@@ -55861,10 +55861,10 @@
         <v>7500.45</v>
       </c>
       <c r="V739" t="n">
-        <v>1.02</v>
+        <v>1.38</v>
       </c>
       <c r="W739" t="n">
-        <v>1.00165158130192</v>
+        <v>1.027203736594576</v>
       </c>
     </row>
     <row r="740">
@@ -56234,7 +56234,7 @@
         <v>1267</v>
       </c>
       <c r="P744" t="n">
-        <v>1122</v>
+        <v>1400</v>
       </c>
       <c r="Q744" t="n">
         <v>1610</v>
@@ -56692,7 +56692,7 @@
         <v>4170</v>
       </c>
       <c r="P750" t="n">
-        <v>3596</v>
+        <v>3820</v>
       </c>
       <c r="Q750" t="n">
         <v>5747</v>
@@ -56771,7 +56771,7 @@
         <v>5858</v>
       </c>
       <c r="P751" t="n">
-        <v>4085</v>
+        <v>4788</v>
       </c>
       <c r="Q751" t="n">
         <v>5858</v>
@@ -56848,7 +56848,7 @@
         <v>5114</v>
       </c>
       <c r="P752" t="n">
-        <v>2184</v>
+        <v>2143</v>
       </c>
       <c r="Q752" t="n">
         <v>5114</v>
@@ -59863,7 +59863,7 @@
         <v>3176</v>
       </c>
       <c r="P793" t="n">
-        <v>0</v>
+        <v>3083</v>
       </c>
       <c r="Q793" t="n">
         <v>3176</v>
@@ -59940,7 +59940,7 @@
         <v>7184</v>
       </c>
       <c r="P794" t="n">
-        <v>1068</v>
+        <v>6765</v>
       </c>
       <c r="Q794" t="n">
         <v>7184</v>
@@ -60017,7 +60017,7 @@
         <v>1241</v>
       </c>
       <c r="P795" t="n">
-        <v>0</v>
+        <v>325</v>
       </c>
       <c r="Q795" t="n">
         <v>1907</v>
@@ -60094,7 +60094,7 @@
         <v>1972</v>
       </c>
       <c r="P796" t="n">
-        <v>0</v>
+        <v>1990</v>
       </c>
       <c r="Q796" t="n">
         <v>2531</v>
@@ -60481,7 +60481,7 @@
         <v>7168</v>
       </c>
       <c r="P801" t="n">
-        <v>5432</v>
+        <v>5629</v>
       </c>
       <c r="Q801" t="n">
         <v>7168</v>
@@ -60953,7 +60953,7 @@
         <v>2103</v>
       </c>
       <c r="P807" t="n">
-        <v>2161</v>
+        <v>2167</v>
       </c>
       <c r="Q807" t="n">
         <v>2316</v>
@@ -61030,13 +61030,13 @@
         <v>2696</v>
       </c>
       <c r="P808" t="n">
-        <v>2860</v>
+        <v>3008</v>
       </c>
       <c r="Q808" t="n">
-        <v>2860</v>
+        <v>3008</v>
       </c>
       <c r="R808" t="n">
-        <v>71.5</v>
+        <v>75.2</v>
       </c>
       <c r="S808" t="n">
         <v>8</v>
@@ -61050,7 +61050,7 @@
         <v>3309.36</v>
       </c>
       <c r="V808" t="n">
-        <v>-13.58</v>
+        <v>-9.109999999999999</v>
       </c>
       <c r="W808" t="inlineStr"/>
     </row>
@@ -61265,13 +61265,13 @@
         <v>5289</v>
       </c>
       <c r="P811" t="n">
-        <v>5571</v>
+        <v>5579</v>
       </c>
       <c r="Q811" t="n">
-        <v>5571</v>
+        <v>5579</v>
       </c>
       <c r="R811" t="n">
-        <v>77.38</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="S811" t="n">
         <v>8</v>
@@ -61285,7 +61285,7 @@
         <v>6089.51</v>
       </c>
       <c r="V811" t="n">
-        <v>-8.51</v>
+        <v>-8.380000000000001</v>
       </c>
       <c r="W811" t="inlineStr"/>
     </row>
@@ -61470,7 +61470,7 @@
         <v>128</v>
       </c>
       <c r="P814" t="n">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="Q814" t="n">
         <v>4173</v>
@@ -62443,7 +62443,7 @@
         <v>3235</v>
       </c>
       <c r="P829" t="n">
-        <v>3276</v>
+        <v>3384</v>
       </c>
       <c r="Q829" t="n">
         <v>3976</v>
@@ -63606,7 +63606,7 @@
         <v>4910</v>
       </c>
       <c r="P844" t="n">
-        <v>4590</v>
+        <v>4716</v>
       </c>
       <c r="Q844" t="n">
         <v>5470</v>
@@ -64228,7 +64228,7 @@
         <v>4278</v>
       </c>
       <c r="P852" t="n">
-        <v>4051</v>
+        <v>4169</v>
       </c>
       <c r="Q852" t="n">
         <v>4278</v>
@@ -65313,7 +65313,7 @@
         <v>6268</v>
       </c>
       <c r="P867" t="n">
-        <v>4852</v>
+        <v>4927</v>
       </c>
       <c r="Q867" t="n">
         <v>6268</v>

</xml_diff>

<commit_message>
Medição Agrupada Atualizada 01/11
</commit_message>
<xml_diff>
--- a/Taxa de Crescimento.xlsx
+++ b/Taxa de Crescimento.xlsx
@@ -677,13 +677,13 @@
         <v>2102</v>
       </c>
       <c r="P3" t="n">
-        <v>2107</v>
+        <v>2131</v>
       </c>
       <c r="Q3" t="n">
-        <v>2107</v>
+        <v>2131</v>
       </c>
       <c r="R3" t="n">
-        <v>33.71</v>
+        <v>34.1</v>
       </c>
       <c r="S3" t="n">
         <v>8</v>
@@ -697,10 +697,10 @@
         <v>1921.26</v>
       </c>
       <c r="V3" t="n">
-        <v>9.67</v>
+        <v>10.92</v>
       </c>
       <c r="W3" t="n">
-        <v>1.208144476913952</v>
+        <v>1.220445957467314</v>
       </c>
     </row>
     <row r="4">
@@ -1369,13 +1369,13 @@
         <v>1036</v>
       </c>
       <c r="P13" t="n">
-        <v>1366</v>
+        <v>1539</v>
       </c>
       <c r="Q13" t="n">
-        <v>1366</v>
+        <v>1539</v>
       </c>
       <c r="R13" t="n">
-        <v>45.53</v>
+        <v>51.3</v>
       </c>
       <c r="S13" t="n">
         <v>8</v>
@@ -1389,9 +1389,11 @@
         <v>1471.72</v>
       </c>
       <c r="V13" t="n">
-        <v>-7.18</v>
-      </c>
-      <c r="W13" t="inlineStr"/>
+        <v>4.57</v>
+      </c>
+      <c r="W13" t="n">
+        <v>1.134992565179017</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1681,7 +1683,7 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>1377</v>
+        <v>1520</v>
       </c>
       <c r="Q17" t="n">
         <v>4925</v>
@@ -1760,7 +1762,7 @@
         <v>14925</v>
       </c>
       <c r="P18" t="n">
-        <v>15662</v>
+        <v>15851</v>
       </c>
       <c r="Q18" t="n">
         <v>28370</v>
@@ -2330,13 +2332,13 @@
         <v>9466</v>
       </c>
       <c r="P26" t="n">
-        <v>9373</v>
+        <v>9471</v>
       </c>
       <c r="Q26" t="n">
-        <v>9466</v>
+        <v>9471</v>
       </c>
       <c r="R26" t="n">
-        <v>75.73</v>
+        <v>75.77</v>
       </c>
       <c r="S26" t="n">
         <v>8</v>
@@ -2350,10 +2352,10 @@
         <v>8440.110000000001</v>
       </c>
       <c r="V26" t="n">
-        <v>12.15</v>
+        <v>12.21</v>
       </c>
       <c r="W26" t="n">
-        <v>1.231349551380652</v>
+        <v>1.231855136280941</v>
       </c>
     </row>
     <row r="27">
@@ -3061,13 +3063,13 @@
         <v>2175</v>
       </c>
       <c r="P37" t="n">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="Q37" t="n">
-        <v>2251</v>
+        <v>2265</v>
       </c>
       <c r="R37" t="n">
-        <v>75.03</v>
+        <v>75.5</v>
       </c>
       <c r="S37" t="n">
         <v>8</v>
@@ -3081,10 +3083,10 @@
         <v>2077.14</v>
       </c>
       <c r="V37" t="n">
-        <v>8.369999999999999</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="W37" t="n">
-        <v>1.19369613630525</v>
+        <v>1.20138084314864</v>
       </c>
     </row>
     <row r="38">
@@ -3811,13 +3813,13 @@
         <v>3477</v>
       </c>
       <c r="P47" t="n">
-        <v>4333</v>
+        <v>4079</v>
       </c>
       <c r="Q47" t="n">
-        <v>4333</v>
+        <v>4079</v>
       </c>
       <c r="R47" t="n">
-        <v>28.89</v>
+        <v>27.19</v>
       </c>
       <c r="S47" t="n">
         <v>8</v>
@@ -3831,7 +3833,7 @@
         <v>4438.47</v>
       </c>
       <c r="V47" t="n">
-        <v>-2.38</v>
+        <v>-8.1</v>
       </c>
       <c r="W47" t="inlineStr"/>
     </row>
@@ -5545,7 +5547,7 @@
         <v>12752</v>
       </c>
       <c r="P71" t="n">
-        <v>11260</v>
+        <v>11158</v>
       </c>
       <c r="Q71" t="n">
         <v>12752</v>
@@ -5622,13 +5624,13 @@
         <v>19630</v>
       </c>
       <c r="P72" t="n">
-        <v>23482</v>
+        <v>24431</v>
       </c>
       <c r="Q72" t="n">
-        <v>23482</v>
+        <v>24431</v>
       </c>
       <c r="R72" t="n">
-        <v>93.93000000000001</v>
+        <v>97.72</v>
       </c>
       <c r="S72" t="n">
         <v>8</v>
@@ -5642,10 +5644,10 @@
         <v>20423.33</v>
       </c>
       <c r="V72" t="n">
-        <v>14.98</v>
+        <v>19.62</v>
       </c>
       <c r="W72" t="n">
-        <v>1.253023793351216</v>
+        <v>1.281518608825801</v>
       </c>
     </row>
     <row r="73">
@@ -7803,7 +7805,7 @@
         <v>3522</v>
       </c>
       <c r="P101" t="n">
-        <v>3348</v>
+        <v>3414</v>
       </c>
       <c r="Q101" t="n">
         <v>3576</v>
@@ -8231,7 +8233,7 @@
         <v>27513</v>
       </c>
       <c r="P107" t="n">
-        <v>12812</v>
+        <v>12281</v>
       </c>
       <c r="Q107" t="n">
         <v>27513</v>
@@ -8310,7 +8312,7 @@
         <v>9607</v>
       </c>
       <c r="P108" t="n">
-        <v>3269</v>
+        <v>2863</v>
       </c>
       <c r="Q108" t="n">
         <v>9607</v>
@@ -10615,13 +10617,13 @@
         <v>22643</v>
       </c>
       <c r="P141" t="n">
-        <v>23453</v>
+        <v>23750</v>
       </c>
       <c r="Q141" t="n">
-        <v>23453</v>
+        <v>23750</v>
       </c>
       <c r="R141" t="n">
-        <v>93.81</v>
+        <v>95</v>
       </c>
       <c r="S141" t="n">
         <v>8</v>
@@ -10635,10 +10637,10 @@
         <v>19800.02</v>
       </c>
       <c r="V141" t="n">
-        <v>18.45</v>
+        <v>19.95</v>
       </c>
       <c r="W141" t="n">
-        <v>1.274969212007679</v>
+        <v>1.283301125039289</v>
       </c>
     </row>
     <row r="142">
@@ -10773,7 +10775,7 @@
         <v>4729</v>
       </c>
       <c r="P143" t="n">
-        <v>5067</v>
+        <v>5101</v>
       </c>
       <c r="Q143" t="n">
         <v>5336</v>
@@ -13264,7 +13266,7 @@
         <v>6068</v>
       </c>
       <c r="P178" t="n">
-        <v>2859</v>
+        <v>2762</v>
       </c>
       <c r="Q178" t="n">
         <v>6068</v>
@@ -16129,7 +16131,7 @@
         <v>13013</v>
       </c>
       <c r="P217" t="n">
-        <v>12581</v>
+        <v>12753</v>
       </c>
       <c r="Q217" t="n">
         <v>13013</v>
@@ -17514,7 +17516,7 @@
         <v>6622</v>
       </c>
       <c r="P236" t="n">
-        <v>5941</v>
+        <v>5991</v>
       </c>
       <c r="Q236" t="n">
         <v>6622</v>
@@ -17826,13 +17828,13 @@
         <v>1844</v>
       </c>
       <c r="P240" t="n">
-        <v>1863</v>
+        <v>1865</v>
       </c>
       <c r="Q240" t="n">
-        <v>1863</v>
+        <v>1865</v>
       </c>
       <c r="R240" t="n">
-        <v>46.39</v>
+        <v>46.44</v>
       </c>
       <c r="S240" t="n">
         <v>8</v>
@@ -17846,10 +17848,10 @@
         <v>1673.48</v>
       </c>
       <c r="V240" t="n">
-        <v>11.32</v>
+        <v>11.44</v>
       </c>
       <c r="W240" t="n">
-        <v>1.22411025306201</v>
+        <v>1.225186403850716</v>
       </c>
     </row>
     <row r="241">
@@ -18217,7 +18219,7 @@
         <v>7078</v>
       </c>
       <c r="P245" t="n">
-        <v>6131</v>
+        <v>5819</v>
       </c>
       <c r="Q245" t="n">
         <v>7078</v>
@@ -18296,7 +18298,7 @@
         <v>7330</v>
       </c>
       <c r="P246" t="n">
-        <v>5759</v>
+        <v>5618</v>
       </c>
       <c r="Q246" t="n">
         <v>7330</v>
@@ -18373,7 +18375,7 @@
         <v>3733</v>
       </c>
       <c r="P247" t="n">
-        <v>2660</v>
+        <v>2643</v>
       </c>
       <c r="Q247" t="n">
         <v>3733</v>
@@ -18450,7 +18452,7 @@
         <v>3899</v>
       </c>
       <c r="P248" t="n">
-        <v>2946</v>
+        <v>2850</v>
       </c>
       <c r="Q248" t="n">
         <v>3899</v>
@@ -18606,7 +18608,7 @@
         <v>4579</v>
       </c>
       <c r="P250" t="n">
-        <v>4327</v>
+        <v>4199</v>
       </c>
       <c r="Q250" t="n">
         <v>4579</v>
@@ -19623,7 +19625,7 @@
         <v>1054</v>
       </c>
       <c r="P263" t="n">
-        <v>1009</v>
+        <v>1038</v>
       </c>
       <c r="Q263" t="n">
         <v>1371</v>
@@ -19779,13 +19781,13 @@
         <v>4353</v>
       </c>
       <c r="P265" t="n">
-        <v>4488</v>
+        <v>4533</v>
       </c>
       <c r="Q265" t="n">
-        <v>4488</v>
+        <v>4533</v>
       </c>
       <c r="R265" t="n">
-        <v>89.41</v>
+        <v>90.31</v>
       </c>
       <c r="S265" t="n">
         <v>8</v>
@@ -19799,10 +19801,10 @@
         <v>3859</v>
       </c>
       <c r="V265" t="n">
-        <v>16.3</v>
+        <v>17.47</v>
       </c>
       <c r="W265" t="n">
-        <v>1.261872958581617</v>
+        <v>1.269183474639503</v>
       </c>
     </row>
     <row r="266">
@@ -20016,13 +20018,13 @@
         <v>6086</v>
       </c>
       <c r="P268" t="n">
-        <v>6309</v>
+        <v>6514</v>
       </c>
       <c r="Q268" t="n">
-        <v>6309</v>
+        <v>6514</v>
       </c>
       <c r="R268" t="n">
-        <v>78.86</v>
+        <v>81.42</v>
       </c>
       <c r="S268" t="n">
         <v>8</v>
@@ -20036,10 +20038,10 @@
         <v>5833.81</v>
       </c>
       <c r="V268" t="n">
-        <v>8.15</v>
+        <v>11.66</v>
       </c>
       <c r="W268" t="n">
-        <v>1.191049471472839</v>
+        <v>1.227132747330455</v>
       </c>
     </row>
     <row r="269">
@@ -20172,13 +20174,13 @@
         <v>2312</v>
       </c>
       <c r="P270" t="n">
-        <v>2398</v>
+        <v>2428</v>
       </c>
       <c r="Q270" t="n">
-        <v>2398</v>
+        <v>2428</v>
       </c>
       <c r="R270" t="n">
-        <v>59.95</v>
+        <v>60.7</v>
       </c>
       <c r="S270" t="n">
         <v>8</v>
@@ -20192,10 +20194,10 @@
         <v>1570.9</v>
       </c>
       <c r="V270" t="n">
-        <v>52.65</v>
+        <v>54.56</v>
       </c>
       <c r="W270" t="n">
-        <v>1.391393161806551</v>
+        <v>1.395531134604049</v>
       </c>
     </row>
     <row r="271">
@@ -20567,7 +20569,7 @@
         <v>4999</v>
       </c>
       <c r="P275" t="n">
-        <v>5018</v>
+        <v>5031</v>
       </c>
       <c r="Q275" t="n">
         <v>5324</v>
@@ -20646,7 +20648,7 @@
         <v>4413</v>
       </c>
       <c r="P276" t="n">
-        <v>4307</v>
+        <v>4400</v>
       </c>
       <c r="Q276" t="n">
         <v>4413</v>
@@ -21161,7 +21163,7 @@
         <v>84</v>
       </c>
       <c r="P283" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="Q283" t="n">
         <v>807</v>
@@ -21238,7 +21240,7 @@
         <v>886</v>
       </c>
       <c r="P284" t="n">
-        <v>914</v>
+        <v>829</v>
       </c>
       <c r="Q284" t="n">
         <v>2450</v>
@@ -22102,13 +22104,13 @@
         <v>2181</v>
       </c>
       <c r="P296" t="n">
-        <v>2249</v>
+        <v>2268</v>
       </c>
       <c r="Q296" t="n">
-        <v>2249</v>
+        <v>2268</v>
       </c>
       <c r="R296" t="n">
-        <v>74.97</v>
+        <v>75.59999999999999</v>
       </c>
       <c r="S296" t="n">
         <v>8</v>
@@ -22122,10 +22124,10 @@
         <v>2083.14</v>
       </c>
       <c r="V296" t="n">
-        <v>7.96</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="W296" t="n">
-        <v>1.188710472869853</v>
+        <v>1.199481723432723</v>
       </c>
     </row>
     <row r="297">
@@ -22181,7 +22183,7 @@
         <v>250</v>
       </c>
       <c r="P297" t="n">
-        <v>253</v>
+        <v>492</v>
       </c>
       <c r="Q297" t="n">
         <v>874</v>
@@ -25107,13 +25109,13 @@
         <v>5311</v>
       </c>
       <c r="P337" t="n">
-        <v>6185</v>
+        <v>6850</v>
       </c>
       <c r="Q337" t="n">
-        <v>6185</v>
+        <v>6850</v>
       </c>
       <c r="R337" t="n">
-        <v>51.54</v>
+        <v>57.08</v>
       </c>
       <c r="S337" t="n">
         <v>8</v>
@@ -25127,10 +25129,10 @@
         <v>4336.29</v>
       </c>
       <c r="V337" t="n">
-        <v>42.63</v>
+        <v>57.97</v>
       </c>
       <c r="W337" t="n">
-        <v>1.367129362810221</v>
+        <v>1.402599269468085</v>
       </c>
     </row>
     <row r="338">
@@ -26190,13 +26192,13 @@
         <v>6030</v>
       </c>
       <c r="P352" t="n">
-        <v>8182</v>
+        <v>7979</v>
       </c>
       <c r="Q352" t="n">
-        <v>8182</v>
+        <v>7979</v>
       </c>
       <c r="R352" t="n">
-        <v>81.5</v>
+        <v>79.48</v>
       </c>
       <c r="S352" t="n">
         <v>8</v>
@@ -26210,10 +26212,10 @@
         <v>5603.53</v>
       </c>
       <c r="V352" t="n">
-        <v>46.02</v>
+        <v>42.39</v>
       </c>
       <c r="W352" t="n">
-        <v>1.375874699173012</v>
+        <v>1.366486308733027</v>
       </c>
     </row>
     <row r="353">
@@ -26346,7 +26348,7 @@
         <v>2641</v>
       </c>
       <c r="P354" t="n">
-        <v>3164</v>
+        <v>2962</v>
       </c>
       <c r="Q354" t="n">
         <v>4698</v>
@@ -27124,13 +27126,13 @@
         <v>2223</v>
       </c>
       <c r="P364" t="n">
-        <v>2106</v>
+        <v>2702</v>
       </c>
       <c r="Q364" t="n">
-        <v>2223</v>
+        <v>2702</v>
       </c>
       <c r="R364" t="n">
-        <v>22.23</v>
+        <v>27.02</v>
       </c>
       <c r="S364" t="n">
         <v>8</v>
@@ -27144,7 +27146,7 @@
         <v>4630.52</v>
       </c>
       <c r="V364" t="n">
-        <v>-51.99</v>
+        <v>-41.65</v>
       </c>
       <c r="W364" t="inlineStr"/>
     </row>
@@ -28143,13 +28145,13 @@
         <v>3531</v>
       </c>
       <c r="P377" t="n">
-        <v>5191</v>
+        <v>5100</v>
       </c>
       <c r="Q377" t="n">
-        <v>5191</v>
+        <v>5100</v>
       </c>
       <c r="R377" t="n">
-        <v>51.91</v>
+        <v>51</v>
       </c>
       <c r="S377" t="n">
         <v>8</v>
@@ -28163,10 +28165,10 @@
         <v>4606.28</v>
       </c>
       <c r="V377" t="n">
-        <v>12.69</v>
+        <v>10.72</v>
       </c>
       <c r="W377" t="n">
-        <v>1.235819760392923</v>
+        <v>1.218567428237834</v>
       </c>
     </row>
     <row r="378">
@@ -28534,7 +28536,7 @@
         <v>5910</v>
       </c>
       <c r="P382" t="n">
-        <v>5163</v>
+        <v>5369</v>
       </c>
       <c r="Q382" t="n">
         <v>5910</v>
@@ -29306,7 +29308,7 @@
         <v>7403</v>
       </c>
       <c r="P392" t="n">
-        <v>5725</v>
+        <v>5593</v>
       </c>
       <c r="Q392" t="n">
         <v>7403</v>
@@ -29383,13 +29385,13 @@
         <v>2485</v>
       </c>
       <c r="P393" t="n">
-        <v>2886</v>
+        <v>2971</v>
       </c>
       <c r="Q393" t="n">
-        <v>2886</v>
+        <v>2971</v>
       </c>
       <c r="R393" t="n">
-        <v>28.86</v>
+        <v>29.71</v>
       </c>
       <c r="S393" t="n">
         <v>8</v>
@@ -29403,7 +29405,7 @@
         <v>3380.62</v>
       </c>
       <c r="V393" t="n">
-        <v>-14.63</v>
+        <v>-12.12</v>
       </c>
       <c r="W393" t="inlineStr"/>
     </row>
@@ -29460,13 +29462,13 @@
         <v>172</v>
       </c>
       <c r="P394" t="n">
-        <v>1020</v>
+        <v>698</v>
       </c>
       <c r="Q394" t="n">
-        <v>1020</v>
+        <v>698</v>
       </c>
       <c r="R394" t="n">
-        <v>10.2</v>
+        <v>6.98</v>
       </c>
       <c r="S394" t="n">
         <v>8</v>
@@ -29480,10 +29482,10 @@
         <v>182.26</v>
       </c>
       <c r="V394" t="n">
-        <v>459.64</v>
+        <v>282.97</v>
       </c>
       <c r="W394" t="n">
-        <v>1.66674112516283</v>
+        <v>1.600706467122624</v>
       </c>
     </row>
     <row r="395">
@@ -29695,13 +29697,13 @@
         <v>1037</v>
       </c>
       <c r="P397" t="n">
-        <v>1486</v>
+        <v>1383</v>
       </c>
       <c r="Q397" t="n">
-        <v>1486</v>
+        <v>1383</v>
       </c>
       <c r="R397" t="n">
-        <v>14.86</v>
+        <v>13.83</v>
       </c>
       <c r="S397" t="n">
         <v>8</v>
@@ -29715,10 +29717,10 @@
         <v>983.04</v>
       </c>
       <c r="V397" t="n">
-        <v>51.16</v>
+        <v>40.69</v>
       </c>
       <c r="W397" t="n">
-        <v>1.388068433753057</v>
+        <v>1.3618333773568</v>
       </c>
     </row>
     <row r="398">
@@ -31298,13 +31300,13 @@
         <v>3854</v>
       </c>
       <c r="P418" t="n">
-        <v>3812</v>
+        <v>4215</v>
       </c>
       <c r="Q418" t="n">
-        <v>3854</v>
+        <v>4215</v>
       </c>
       <c r="R418" t="n">
-        <v>38.54</v>
+        <v>42.15</v>
       </c>
       <c r="S418" t="n">
         <v>8</v>
@@ -31318,7 +31320,7 @@
         <v>7407.03</v>
       </c>
       <c r="V418" t="n">
-        <v>-47.97</v>
+        <v>-43.09</v>
       </c>
       <c r="W418" t="inlineStr"/>
     </row>
@@ -33792,13 +33794,13 @@
         <v>4704</v>
       </c>
       <c r="P450" t="n">
-        <v>5708</v>
+        <v>5716</v>
       </c>
       <c r="Q450" t="n">
-        <v>5708</v>
+        <v>5716</v>
       </c>
       <c r="R450" t="n">
-        <v>56.86</v>
+        <v>56.94</v>
       </c>
       <c r="S450" t="n">
         <v>8</v>
@@ -33812,7 +33814,7 @@
         <v>5969.77</v>
       </c>
       <c r="V450" t="n">
-        <v>-4.38</v>
+        <v>-4.25</v>
       </c>
       <c r="W450" t="inlineStr"/>
     </row>
@@ -33948,13 +33950,13 @@
         <v>4114</v>
       </c>
       <c r="P452" t="n">
-        <v>6442</v>
+        <v>6837</v>
       </c>
       <c r="Q452" t="n">
-        <v>6442</v>
+        <v>6837</v>
       </c>
       <c r="R452" t="n">
-        <v>64.42</v>
+        <v>68.37</v>
       </c>
       <c r="S452" t="n">
         <v>8</v>
@@ -33968,10 +33970,10 @@
         <v>4416.41</v>
       </c>
       <c r="V452" t="n">
-        <v>45.87</v>
+        <v>54.81</v>
       </c>
       <c r="W452" t="n">
-        <v>1.375500423197763</v>
+        <v>1.396062892028175</v>
       </c>
     </row>
     <row r="453">
@@ -35498,13 +35500,13 @@
         <v>2969</v>
       </c>
       <c r="P472" t="n">
-        <v>3423</v>
+        <v>5619</v>
       </c>
       <c r="Q472" t="n">
-        <v>3423</v>
+        <v>5619</v>
       </c>
       <c r="R472" t="n">
-        <v>42.79</v>
+        <v>70.23999999999999</v>
       </c>
       <c r="S472" t="n">
         <v>8</v>
@@ -35518,7 +35520,7 @@
         <v>5789.98</v>
       </c>
       <c r="V472" t="n">
-        <v>-40.88</v>
+        <v>-2.95</v>
       </c>
       <c r="W472" t="inlineStr"/>
     </row>
@@ -35731,13 +35733,13 @@
         <v>5733</v>
       </c>
       <c r="P475" t="n">
-        <v>6132</v>
+        <v>7796</v>
       </c>
       <c r="Q475" t="n">
-        <v>6132</v>
+        <v>7796</v>
       </c>
       <c r="R475" t="n">
-        <v>61.32</v>
+        <v>77.95999999999999</v>
       </c>
       <c r="S475" t="n">
         <v>8</v>
@@ -35751,9 +35753,11 @@
         <v>6786.37</v>
       </c>
       <c r="V475" t="n">
-        <v>-9.640000000000001</v>
-      </c>
-      <c r="W475" t="inlineStr"/>
+        <v>14.88</v>
+      </c>
+      <c r="W475" t="n">
+        <v>1.252324597746059</v>
+      </c>
     </row>
     <row r="476">
       <c r="A476" t="inlineStr">
@@ -38537,13 +38541,13 @@
         <v>7115</v>
       </c>
       <c r="P511" t="n">
-        <v>7535</v>
+        <v>8280</v>
       </c>
       <c r="Q511" t="n">
-        <v>8169</v>
+        <v>8280</v>
       </c>
       <c r="R511" t="n">
-        <v>81.69</v>
+        <v>82.8</v>
       </c>
       <c r="S511" t="n">
         <v>8</v>
@@ -38557,7 +38561,7 @@
         <v>9717.57</v>
       </c>
       <c r="V511" t="n">
-        <v>-15.94</v>
+        <v>-14.79</v>
       </c>
       <c r="W511" t="inlineStr"/>
     </row>
@@ -39311,13 +39315,13 @@
         <v>4667</v>
       </c>
       <c r="P521" t="n">
-        <v>4666</v>
+        <v>4816</v>
       </c>
       <c r="Q521" t="n">
-        <v>4712</v>
+        <v>4816</v>
       </c>
       <c r="R521" t="n">
-        <v>47.12</v>
+        <v>48.16</v>
       </c>
       <c r="S521" t="n">
         <v>8</v>
@@ -39331,10 +39335,10 @@
         <v>4539.56</v>
       </c>
       <c r="V521" t="n">
-        <v>3.8</v>
+        <v>6.09</v>
       </c>
       <c r="W521" t="n">
-        <v>1.11767438985762</v>
+        <v>1.162478085141094</v>
       </c>
     </row>
     <row r="522">
@@ -41160,7 +41164,7 @@
         <v>2804</v>
       </c>
       <c r="P546" t="n">
-        <v>711</v>
+        <v>688</v>
       </c>
       <c r="Q546" t="n">
         <v>5012</v>
@@ -41237,7 +41241,7 @@
         <v>5417</v>
       </c>
       <c r="P547" t="n">
-        <v>2415</v>
+        <v>2274</v>
       </c>
       <c r="Q547" t="n">
         <v>6510</v>
@@ -41472,7 +41476,7 @@
         <v>6600</v>
       </c>
       <c r="P550" t="n">
-        <v>5751</v>
+        <v>5188</v>
       </c>
       <c r="Q550" t="n">
         <v>8472</v>
@@ -41551,7 +41555,7 @@
         <v>3233</v>
       </c>
       <c r="P551" t="n">
-        <v>2219</v>
+        <v>742</v>
       </c>
       <c r="Q551" t="n">
         <v>3752</v>
@@ -41979,7 +41983,7 @@
         <v>529</v>
       </c>
       <c r="P557" t="n">
-        <v>454</v>
+        <v>435</v>
       </c>
       <c r="Q557" t="n">
         <v>603</v>
@@ -42156,13 +42160,13 @@
         <v>1904</v>
       </c>
       <c r="P560" t="n">
-        <v>3456</v>
+        <v>3563</v>
       </c>
       <c r="Q560" t="n">
-        <v>3456</v>
+        <v>3563</v>
       </c>
       <c r="R560" t="n">
-        <v>17.28</v>
+        <v>17.82</v>
       </c>
       <c r="S560" t="n">
         <v>8</v>
@@ -42176,7 +42180,7 @@
         <v>4921.4</v>
       </c>
       <c r="V560" t="n">
-        <v>-29.78</v>
+        <v>-27.6</v>
       </c>
       <c r="W560" t="inlineStr"/>
     </row>
@@ -43115,7 +43119,7 @@
         <v>3766</v>
       </c>
       <c r="P573" t="n">
-        <v>3008</v>
+        <v>2695</v>
       </c>
       <c r="Q573" t="n">
         <v>3836</v>
@@ -43350,13 +43354,13 @@
         <v>4368</v>
       </c>
       <c r="P576" t="n">
-        <v>4456</v>
+        <v>4606</v>
       </c>
       <c r="Q576" t="n">
-        <v>4456</v>
+        <v>4606</v>
       </c>
       <c r="R576" t="n">
-        <v>67.55</v>
+        <v>69.81999999999999</v>
       </c>
       <c r="S576" t="n">
         <v>8</v>
@@ -43370,7 +43374,7 @@
         <v>5866.41</v>
       </c>
       <c r="V576" t="n">
-        <v>-24.04</v>
+        <v>-21.49</v>
       </c>
       <c r="W576" t="inlineStr"/>
     </row>
@@ -44793,7 +44797,7 @@
         <v>398</v>
       </c>
       <c r="P595" t="n">
-        <v>167</v>
+        <v>92</v>
       </c>
       <c r="Q595" t="n">
         <v>398</v>
@@ -46203,7 +46207,7 @@
         <v>3274</v>
       </c>
       <c r="P613" t="n">
-        <v>2532</v>
+        <v>2933</v>
       </c>
       <c r="Q613" t="n">
         <v>3274</v>
@@ -48001,13 +48005,13 @@
         <v>447</v>
       </c>
       <c r="P637" t="n">
-        <v>687</v>
+        <v>942</v>
       </c>
       <c r="Q637" t="n">
-        <v>687</v>
+        <v>942</v>
       </c>
       <c r="R637" t="n">
-        <v>11.45</v>
+        <v>15.7</v>
       </c>
       <c r="S637" t="n">
         <v>8</v>
@@ -48021,7 +48025,7 @@
         <v>964.63</v>
       </c>
       <c r="V637" t="n">
-        <v>-28.78</v>
+        <v>-2.35</v>
       </c>
       <c r="W637" t="inlineStr"/>
     </row>
@@ -48315,7 +48319,7 @@
         <v>7248</v>
       </c>
       <c r="P641" t="n">
-        <v>4823</v>
+        <v>4412</v>
       </c>
       <c r="Q641" t="n">
         <v>9088</v>
@@ -49403,7 +49407,7 @@
         <v>2179</v>
       </c>
       <c r="P655" t="n">
-        <v>2151</v>
+        <v>2780</v>
       </c>
       <c r="Q655" t="n">
         <v>2801</v>
@@ -51010,13 +51014,13 @@
         <v>2439</v>
       </c>
       <c r="P676" t="n">
-        <v>3098</v>
+        <v>3083</v>
       </c>
       <c r="Q676" t="n">
-        <v>3098</v>
+        <v>3083</v>
       </c>
       <c r="R676" t="n">
-        <v>25.82</v>
+        <v>25.69</v>
       </c>
       <c r="S676" t="n">
         <v>8</v>
@@ -51030,7 +51034,7 @@
         <v>4555.14</v>
       </c>
       <c r="V676" t="n">
-        <v>-31.99</v>
+        <v>-32.32</v>
       </c>
       <c r="W676" t="inlineStr"/>
     </row>
@@ -52119,13 +52123,13 @@
         <v>372</v>
       </c>
       <c r="P691" t="n">
-        <v>687</v>
+        <v>932</v>
       </c>
       <c r="Q691" t="n">
-        <v>687</v>
+        <v>932</v>
       </c>
       <c r="R691" t="n">
-        <v>15.98</v>
+        <v>21.67</v>
       </c>
       <c r="S691" t="n">
         <v>8</v>
@@ -52139,7 +52143,7 @@
         <v>1851.79</v>
       </c>
       <c r="V691" t="n">
-        <v>-62.9</v>
+        <v>-49.67</v>
       </c>
       <c r="W691" t="inlineStr"/>
     </row>
@@ -53124,13 +53128,13 @@
         <v>266</v>
       </c>
       <c r="P704" t="n">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="Q704" t="n">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="R704" t="n">
-        <v>6.9</v>
+        <v>7.02</v>
       </c>
       <c r="S704" t="n">
         <v>8</v>
@@ -53144,7 +53148,7 @@
         <v>285.39</v>
       </c>
       <c r="V704" t="n">
-        <v>-3.29</v>
+        <v>-1.54</v>
       </c>
       <c r="W704" t="inlineStr"/>
     </row>
@@ -53357,7 +53361,7 @@
         <v>400</v>
       </c>
       <c r="P707" t="n">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="Q707" t="n">
         <v>410</v>
@@ -53434,7 +53438,7 @@
         <v>3176</v>
       </c>
       <c r="P708" t="n">
-        <v>1030</v>
+        <v>1082</v>
       </c>
       <c r="Q708" t="n">
         <v>3176</v>
@@ -53902,7 +53906,7 @@
         <v>4</v>
       </c>
       <c r="P714" t="n">
-        <v>-56</v>
+        <v>-50</v>
       </c>
       <c r="Q714" t="n">
         <v>4528</v>
@@ -54370,13 +54374,13 @@
         <v>1355</v>
       </c>
       <c r="P720" t="n">
-        <v>1334</v>
+        <v>1627</v>
       </c>
       <c r="Q720" t="n">
-        <v>1486</v>
+        <v>1627</v>
       </c>
       <c r="R720" t="n">
-        <v>14.8</v>
+        <v>16.21</v>
       </c>
       <c r="S720" t="n">
         <v>8</v>
@@ -54390,7 +54394,7 @@
         <v>4501.56</v>
       </c>
       <c r="V720" t="n">
-        <v>-66.98999999999999</v>
+        <v>-63.86</v>
       </c>
       <c r="W720" t="inlineStr"/>
     </row>
@@ -55454,7 +55458,7 @@
         <v>6867</v>
       </c>
       <c r="P734" t="n">
-        <v>6370</v>
+        <v>6562</v>
       </c>
       <c r="Q734" t="n">
         <v>7742</v>
@@ -56155,7 +56159,7 @@
         <v>8830</v>
       </c>
       <c r="P743" t="n">
-        <v>6506</v>
+        <v>5581</v>
       </c>
       <c r="Q743" t="n">
         <v>8830</v>
@@ -56848,7 +56852,7 @@
         <v>5114</v>
       </c>
       <c r="P752" t="n">
-        <v>1917</v>
+        <v>1882</v>
       </c>
       <c r="Q752" t="n">
         <v>5114</v>
@@ -56921,7 +56925,7 @@
         <v>1154</v>
       </c>
       <c r="P753" t="n">
-        <v>910</v>
+        <v>877</v>
       </c>
       <c r="Q753" t="n">
         <v>1431</v>
@@ -57150,13 +57154,13 @@
         <v>1934</v>
       </c>
       <c r="P756" t="n">
-        <v>3412</v>
+        <v>3352</v>
       </c>
       <c r="Q756" t="n">
-        <v>3412</v>
+        <v>3352</v>
       </c>
       <c r="R756" t="n">
-        <v>42.65</v>
+        <v>41.9</v>
       </c>
       <c r="S756" t="n">
         <v>8</v>
@@ -57170,10 +57174,10 @@
         <v>2448.7</v>
       </c>
       <c r="V756" t="n">
-        <v>39.34</v>
+        <v>36.89</v>
       </c>
       <c r="W756" t="n">
-        <v>1.358009671633811</v>
+        <v>1.350752317292871</v>
       </c>
     </row>
     <row r="757">
@@ -62676,13 +62680,13 @@
         <v>7806</v>
       </c>
       <c r="P832" t="n">
-        <v>7480</v>
+        <v>9400</v>
       </c>
       <c r="Q832" t="n">
-        <v>7806</v>
+        <v>9400</v>
       </c>
       <c r="R832" t="n">
-        <v>65.05</v>
+        <v>78.33</v>
       </c>
       <c r="S832" t="n">
         <v>8</v>
@@ -62696,10 +62700,10 @@
         <v>4603.66</v>
       </c>
       <c r="V832" t="n">
-        <v>69.56</v>
+        <v>104.19</v>
       </c>
       <c r="W832" t="n">
-        <v>1.424065497627815</v>
+        <v>1.472828467557885</v>
       </c>
     </row>
     <row r="833">
@@ -62911,13 +62915,13 @@
         <v>1722</v>
       </c>
       <c r="P835" t="n">
-        <v>1891</v>
+        <v>1749</v>
       </c>
       <c r="Q835" t="n">
-        <v>1891</v>
+        <v>1749</v>
       </c>
       <c r="R835" t="n">
-        <v>21.01</v>
+        <v>19.43</v>
       </c>
       <c r="S835" t="n">
         <v>8</v>
@@ -62931,7 +62935,7 @@
         <v>3162.28</v>
       </c>
       <c r="V835" t="n">
-        <v>-40.2</v>
+        <v>-44.69</v>
       </c>
       <c r="W835" t="inlineStr"/>
     </row>
@@ -65627,7 +65631,7 @@
         <v>5274</v>
       </c>
       <c r="P871" t="n">
-        <v>3737</v>
+        <v>3760</v>
       </c>
       <c r="Q871" t="n">
         <v>8343</v>

</xml_diff>